<commit_message>
docs: Test and static analysis reports for SDK 8.6
Added test reports for SDK 8.6 generated with new TPER-Qmetry script.
Traceability matrix are not being included as the tool doesn't support
it yet, so previous traceability matrix reports are being removed as
they are for previous release.

Static analysis report generated with new SCAR script is also being
included.

Signed-off-by: Misael Lopez Cruz <misael.lopez@ti.com>
</commit_message>
<xml_diff>
--- a/docs/misrac/ethfw_SA_Report.xlsx
+++ b/docs/misrac/ethfw_SA_Report.xlsx
@@ -26,7 +26,7 @@
     <sheet name="Klocwork Project Modules" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="10" name="_xlnm._FilterDatabase">'Raw Issue Details'!$A$1:$T$7</definedName>
+    <definedName hidden="1" localSheetId="10" name="_xlnm._FilterDatabase">'Raw Issue Details'!$A$1:$T$4</definedName>
     <definedName hidden="1" localSheetId="11" name="_xlnm._FilterDatabase">'Guideline Enforcement Plan'!$A$1:$I$255</definedName>
     <definedName hidden="1" localSheetId="14" name="_xlnm._FilterDatabase">'Active Deviation Permits'!$A$1:$J$67</definedName>
     <definedName hidden="1" localSheetId="15" name="_xlnm._FilterDatabase">'Taxonomy Checkers'!$A$1:$F$1126</definedName>
@@ -38,7 +38,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="16"/>
     </font>
     <font>
       <color rgb="00ffffff"/>
@@ -130,15 +134,24 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf applyAlignment="1" borderId="1" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf applyAlignment="1" borderId="1" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf applyAlignment="1" borderId="1" fillId="5" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
@@ -165,7 +178,7 @@
     <xf applyAlignment="1" borderId="0" fillId="7" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="11" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="1" fillId="11" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf applyAlignment="1" borderId="1" fillId="10" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
@@ -468,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="10"/>
@@ -479,276 +492,303 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>TI Information - Selective Disclosure</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="n"/>
+      <c r="C1" s="3" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Copyright (C) 2023 Texas Instruments Incorporated</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="5" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
           <t>Sheet No.</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Purpose</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Table of Contents</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Provides an overview of the contents of the complete report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Script Input Parameters</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Displays the input parameters provided to generate this report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Klocwork Build Configuration</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Provides an overview on the build in the Klocwork project for which this report has been generated.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>MISRA Summary by Metrics</t>
+          <t>Table of Contents</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Provides a short summary which was earlier part of HIS Summary by Metrics report in FoQus-generated HIS Reports.</t>
+          <t>Provides an overview of the contents of the complete report.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>MISRA Summary by Severity</t>
+          <t>Script Input Parameters</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Provides MISRA Summary Report by Severity on the issues identified.</t>
+          <t>Displays the input parameters provided to generate this report.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>MISRA Summary by Modules</t>
+          <t>Klocwork Build Configuration</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Provides MISRA Summary Report by Modules. These modules are defined in the Klocwork project. Each module can have multiple file paths included in it.</t>
+          <t>Provides an overview on the build in the Klocwork project for which this report has been generated.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>HIS Summary by Metrics</t>
+          <t>MISRA Summary by Metrics</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Provides HIS Summary Report by Metrics.</t>
+          <t>Provides a short summary which was earlier part of HIS Summary by Metrics report in FoQus-generated HIS Reports.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>HIS Summary by Modules</t>
+          <t>MISRA Summary by Severity</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Provides HIS Summary Report by Modules for each HIS Metric.</t>
+          <t>Provides MISRA Summary Report by Severity on the issues identified.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SA Summary by Severity</t>
+          <t>MISRA Summary by Modules</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Provides Static Analysis (SA) Summary Report by Severity on the issues identified.</t>
+          <t>Provides MISRA Summary Report by Modules. These modules are defined in the Klocwork project. Each module can have multiple file paths included in it.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SA Summary by Modules</t>
+          <t>HIS Summary by Metrics</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Provides Static Analysis (SA) Summary Report by Modules. These modules are defined in the Klocwork project. Each module can have multiple file paths included in it.</t>
+          <t>Provides HIS Summary Report by Metrics.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Raw Issue Details</t>
+          <t>HIS Summary by Modules</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Provides raw issue details from Klocwork. If you provided MISRA taxonomy as input parameter, it will also consist of Waiver details.</t>
+          <t>Provides HIS Summary Report by Modules for each HIS Metric.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Guideline Enforcement Plan</t>
+          <t>SA Summary by Severity</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Provides MISRA Guideline Enforcement Plan.</t>
+          <t>Provides Static Analysis (SA) Summary Report by Severity on the issues identified.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Deviation Summary by Type &amp; Category</t>
+          <t>SA Summary by Modules</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Provides MISRA Active Deviation Summary by Category for Deviation Types.</t>
+          <t>Provides Static Analysis (SA) Summary Report by Modules. These modules are defined in the Klocwork project. Each module can have multiple file paths included in it.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Deviation Summary by Classification</t>
+          <t>Raw Issue Details</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Provides MISRA Active Deviation Summary by Classification</t>
+          <t>Provides raw issue details from Klocwork. If you provided MISRA taxonomy as input parameter, it will also consist of Waiver details.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Active Deviation Permits</t>
+          <t>Guideline Enforcement Plan</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Provides MISRA Active Deviation Permit details from Jira including both EP-wide and project-specific Waivers.</t>
+          <t>Provides MISRA Guideline Enforcement Plan.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Taxonomy Checkers</t>
+          <t>Deviation Summary by Type &amp; Category</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Provides the list of checkers from the taxonomy/taxonomies in Klocwork.</t>
+          <t>Provides MISRA Active Deviation Summary by Category for Deviation Types.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Deviation Summary by Classification</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Provides MISRA Active Deviation Summary by Classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Active Deviation Permits</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Provides MISRA Active Deviation Permit details from Jira including both EP-wide and project-specific Waivers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Taxonomy Checkers</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Provides the list of checkers from the taxonomy/taxonomies in Klocwork.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Klocwork Project Modules</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Provides the list of modules defined the Klocwork project along with the file paths included in them.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
@@ -778,74 +818,74 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Module name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>State: New</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>State: New AND need to be Analyzed or Fixed</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>State: Existing</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>State: Existing AND need to be Analyzed or Fixed</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Status: Analyze</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Status: Ignore</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Status: Not a Problem</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Status: Defer</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Status: Fix</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Status: Fix in Next Release</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>Status: Fix in Later Release</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>Status: Filter</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>EthFw</t>
         </is>
@@ -888,45 +928,45 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="B3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="11" t="n">
+      <c r="B3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="11" t="n">
+      <c r="E3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="H3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="11" t="n">
+      <c r="H3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -941,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="18"/>
@@ -967,102 +1007,102 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>comment</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>file</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>line</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>message</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="15" t="inlineStr">
         <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="J1" s="12" t="inlineStr">
+      <c r="J1" s="15" t="inlineStr">
         <is>
           <t>severityCode</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>taxonomyName</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="O1" s="8" t="inlineStr">
+      <c r="O1" s="11" t="inlineStr">
         <is>
           <t>Waiver ID</t>
         </is>
       </c>
-      <c r="P1" s="8" t="inlineStr">
+      <c r="P1" s="11" t="inlineStr">
         <is>
           <t>Waiver Classification</t>
         </is>
       </c>
-      <c r="Q1" s="8" t="inlineStr">
+      <c r="Q1" s="11" t="inlineStr">
         <is>
           <t>Deviation Type</t>
         </is>
       </c>
-      <c r="R1" s="12" t="inlineStr">
+      <c r="R1" s="15" t="inlineStr">
         <is>
           <t>MISRA Rule</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="6" t="inlineStr">
         <is>
           <t>module</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="6" t="inlineStr">
         <is>
           <t>Waiver ID/ Comment Validation</t>
         </is>
@@ -1088,7 +1128,7 @@
         <v>148377</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1366</v>
+        <v>1376</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
@@ -1129,7 +1169,7 @@
         </is>
       </c>
       <c r="N2" s="3">
-        <f>HYPERLINK("https://klocwork.india.ti.com:443/review/insight-review.html#issuedetails_goto:problemid=148377,project=ETHSWITCHFW,searchquery=taxonomy:'' build:KW_Build_Label_Dec_04_2022_12_26_AM grouping:off status:'Not a Problem',Ignore severity:'Error','Critical'","KW Issue Link")</f>
+        <f>HYPERLINK("https://klocwork.india.ti.com:443/review/insight-review.html#issuedetails_goto:problemid=148377,project=ETHSWITCHFW,searchquery=taxonomy:'' build:KW_Build_Label_Feb_15_2023_12_21_PM grouping:off status:'Not a Problem',Ignore severity:'Error','Critical' module:+'EthFw'","KW Issue Link")</f>
         <v/>
       </c>
       <c r="O2" s="3" t="inlineStr"/>
@@ -1146,33 +1186,33 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ABV.STACK</t>
+          <t>RH.LEAK</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Specific EnetTypes are checked in lines 487-488 that would prevent the buffer overflow from happening.</t>
+          <t>Permitted as per deviation record PSDKRA_SA_DR_011.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>/data/adasuser_bangvideoapps02/ethfw_jenkin_build/kw_build/ethfw/ethfw/src/ethfw.c</t>
+          <t>/data/adasuser_bangvideoapps02/ethfw_jenkin_build/kw_build/ethfw/utils/console_io/src/app_log_printf_ticgt_rtos.c</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>423723</v>
+        <v>1086257</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1159</v>
+        <v>243</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Array 'gMcmObj' of size 7 may use index value(s) 0..7</t>
+          <t>Resource acquired to 'freopen("appLog:", "w",  ( &amp;_ftable[1] ) )' at line 243 may be lost here.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>EthFw_initMcm</t>
+          <t>appLogCioInit</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -1182,11 +1222,11 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Error</t>
         </is>
       </c>
       <c r="J3" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
@@ -1195,7 +1235,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Not a Problem</t>
+          <t>Ignore</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -1204,7 +1244,7 @@
         </is>
       </c>
       <c r="N3" s="3">
-        <f>HYPERLINK("https://klocwork.india.ti.com:443/review/insight-review.html#issuedetails_goto:problemid=423723,project=ETHSWITCHFW,searchquery=taxonomy:'' build:KW_Build_Label_Dec_04_2022_12_26_AM grouping:off status:'Not a Problem',Ignore severity:'Error','Critical'","KW Issue Link")</f>
+        <f>HYPERLINK("https://klocwork.india.ti.com:443/review/insight-review.html#issuedetails_goto:problemid=1086257,project=ETHSWITCHFW,searchquery=taxonomy:'' build:KW_Build_Label_Feb_15_2023_12_21_PM grouping:off status:'Not a Problem',Ignore severity:'Error','Critical' module:+'EthFw'","KW Issue Link")</f>
         <v/>
       </c>
       <c r="O3" s="3" t="inlineStr"/>
@@ -1213,7 +1253,7 @@
       <c r="R3" s="3" t="inlineStr"/>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>*default*</t>
+          <t>*default*, EthFw</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr"/>
@@ -1226,19 +1266,19 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>This is called by EthFw which runs forever and is not expected to be terminated.</t>
+          <t>Permitted as per deviation record PSDKRA_SA_DR_006.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>/data/adasuser_bangvideoapps02/ethfw_jenkin_build/kw_build/pdk/packages/ti/drv/enet/enet_cfgserver/enet_cfgserver.c</t>
+          <t>/data/adasuser_bangvideoapps02/ethfw_jenkin_build/kw_build/ethfw/apps/app_remoteswitchcfg_server/mcu_2_0/main.c</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>700252</v>
+        <v>1087079</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>442</v>
+        <v>1152</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
@@ -1247,7 +1287,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>EnetCfgServer_networkTask</t>
+          <t>EthApp_traceBufFlush</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -1270,7 +1310,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Not a Problem</t>
+          <t>Ignore</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -1279,7 +1319,7 @@
         </is>
       </c>
       <c r="N4" s="3">
-        <f>HYPERLINK("https://klocwork.india.ti.com:443/review/insight-review.html#issuedetails_goto:problemid=700252,project=ETHSWITCHFW,searchquery=taxonomy:'' build:KW_Build_Label_Dec_04_2022_12_26_AM grouping:off status:'Not a Problem',Ignore severity:'Error','Critical'","KW Issue Link")</f>
+        <f>HYPERLINK("https://klocwork.india.ti.com:443/review/insight-review.html#issuedetails_goto:problemid=1087079,project=ETHSWITCHFW,searchquery=taxonomy:'' build:KW_Build_Label_Feb_15_2023_12_21_PM grouping:off status:'Not a Problem',Ignore severity:'Error','Critical' module:+'EthFw'","KW Issue Link")</f>
         <v/>
       </c>
       <c r="O4" s="3" t="inlineStr"/>
@@ -1288,238 +1328,13 @@
       <c r="R4" s="3" t="inlineStr"/>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>*default*</t>
+          <t>*default*, EthFw</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr"/>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>INFINITE_LOOP.LOCAL</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>This is called by EthFw which runs forever and is not expected to be terminated.</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>/data/adasuser_bangvideoapps02/ethfw_jenkin_build/kw_build/pdk/packages/ti/drv/enet/enet_cfgserver/enet_cfgserver.c</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>700253</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>496</v>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Infinite loop</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>EnetCfgServer_dispatcherTask</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>unowned</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Error</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>Not a Problem</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>C and C++</t>
-        </is>
-      </c>
-      <c r="N5" s="3">
-        <f>HYPERLINK("https://klocwork.india.ti.com:443/review/insight-review.html#issuedetails_goto:problemid=700253,project=ETHSWITCHFW,searchquery=taxonomy:'' build:KW_Build_Label_Dec_04_2022_12_26_AM grouping:off status:'Not a Problem',Ignore severity:'Error','Critical'","KW Issue Link")</f>
-        <v/>
-      </c>
-      <c r="O5" s="3" t="inlineStr"/>
-      <c r="P5" s="3" t="inlineStr"/>
-      <c r="Q5" s="3" t="inlineStr"/>
-      <c r="R5" s="3" t="inlineStr"/>
-      <c r="S5" s="3" t="inlineStr">
-        <is>
-          <t>*default*</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>RH.LEAK</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Permitted as per deviation record PSDKRA_SA_DR_011.</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>/data/adasuser_bangvideoapps02/ethfw_jenkin_build/kw_build/ethfw/utils/console_io/src/app_log_printf_ticgt_rtos.c</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>1086257</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>243</v>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Resource acquired to 'freopen("appLog:", "w",  ( &amp;_ftable[1] ) )' at line 243 may be lost here.</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>appLogCioInit</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>unowned</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>Error</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>Ignore</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>C and C++</t>
-        </is>
-      </c>
-      <c r="N6" s="3">
-        <f>HYPERLINK("https://klocwork.india.ti.com:443/review/insight-review.html#issuedetails_goto:problemid=1086257,project=ETHSWITCHFW,searchquery=taxonomy:'' build:KW_Build_Label_Dec_04_2022_12_26_AM grouping:off status:'Not a Problem',Ignore severity:'Error','Critical'","KW Issue Link")</f>
-        <v/>
-      </c>
-      <c r="O6" s="3" t="inlineStr"/>
-      <c r="P6" s="3" t="inlineStr"/>
-      <c r="Q6" s="3" t="inlineStr"/>
-      <c r="R6" s="3" t="inlineStr"/>
-      <c r="S6" s="3" t="inlineStr">
-        <is>
-          <t>*default*, EthFw</t>
-        </is>
-      </c>
-      <c r="T6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>INFINITE_LOOP.LOCAL</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Permitted as per deviation record PSDKRA_SA_DR_006.</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>/data/adasuser_bangvideoapps02/ethfw_jenkin_build/kw_build/ethfw/apps/app_remoteswitchcfg_server/mcu_2_0/main.c</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>1087079</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>1133</v>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Infinite loop</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>EthApp_traceBufFlush</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>unowned</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>Error</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>Ignore</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>C and C++</t>
-        </is>
-      </c>
-      <c r="N7" s="3">
-        <f>HYPERLINK("https://klocwork.india.ti.com:443/review/insight-review.html#issuedetails_goto:problemid=1087079,project=ETHSWITCHFW,searchquery=taxonomy:'' build:KW_Build_Label_Dec_04_2022_12_26_AM grouping:off status:'Not a Problem',Ignore severity:'Error','Critical'","KW Issue Link")</f>
-        <v/>
-      </c>
-      <c r="O7" s="3" t="inlineStr"/>
-      <c r="P7" s="3" t="inlineStr"/>
-      <c r="Q7" s="3" t="inlineStr"/>
-      <c r="R7" s="3" t="inlineStr"/>
-      <c r="S7" s="3" t="inlineStr">
-        <is>
-          <t>*default*, EthFw</t>
-        </is>
-      </c>
-      <c r="T7" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:T7"/>
+  <autoFilter ref="A1:T4"/>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
@@ -1545,47 +1360,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>MISRA Rule</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Decidable?</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>Rule Description</t>
         </is>
       </c>
-      <c r="E1" s="13" t="inlineStr">
+      <c r="E1" s="16" t="inlineStr">
         <is>
           <t>Checker Code</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
+      <c r="F1" s="16" t="inlineStr">
         <is>
           <t>Alternate Checker - Compiler/Linker</t>
         </is>
       </c>
-      <c r="G1" s="13" t="inlineStr">
+      <c r="G1" s="16" t="inlineStr">
         <is>
           <t>Alternate Checker - Manual Review</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Waiver ID</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Waiver Link</t>
         </is>
@@ -9782,17 +9597,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Deviation Type | Category</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Advisory</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
@@ -9838,15 +9653,15 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Total Active Deviation Permits</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="14" t="n">
         <v>40</v>
       </c>
     </row>
@@ -9869,12 +9684,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Waiver Classification</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>No. of Active Deviation Permits</t>
         </is>
@@ -9961,12 +9776,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Total Active Deviation Permits</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="14" t="n">
         <v>66</v>
       </c>
     </row>
@@ -9997,52 +9812,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Waiver ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Waiver Link</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Deviation Type</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Waiver Classification</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Waiver Use-Case</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
+      <c r="F1" s="16" t="inlineStr">
         <is>
           <t>MISRA Rule</t>
         </is>
       </c>
-      <c r="G1" s="13" t="inlineStr">
+      <c r="G1" s="16" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="H1" s="13" t="inlineStr">
+      <c r="H1" s="16" t="inlineStr">
         <is>
           <t>Decidable?</t>
         </is>
       </c>
-      <c r="I1" s="13" t="inlineStr">
+      <c r="I1" s="16" t="inlineStr">
         <is>
           <t>Rule Description</t>
         </is>
       </c>
-      <c r="J1" s="13" t="inlineStr">
+      <c r="J1" s="16" t="inlineStr">
         <is>
           <t>Checker Code</t>
         </is>
@@ -14565,32 +14380,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>supportLevel</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Taxonomy Name</t>
         </is>
@@ -43794,12 +43609,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>paths</t>
         </is>
@@ -43840,32 +43655,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Klocwork Project</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Taxonomy</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Advanced Query</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Jira Project Key</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Report generated on</t>
         </is>
@@ -43880,12 +43695,12 @@
       <c r="B2" s="3" t="inlineStr"/>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>KW_Build_Label_Dec_04_2022_12_26_AM</t>
+          <t>KW_Build_Label_Feb_15_2023_12_21_PM</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>status:'Not a Problem',Ignore severity:'Error','Critical'</t>
+          <t>status:'Not a Problem',Ignore severity:'Error','Critical' module:+'EthFw'</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -43895,7 +43710,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>2022-12-08 23:22:46.565546-06:00 CDT</t>
+          <t>2023-02-15 02:47:07.084259-06:00 CDT</t>
         </is>
       </c>
     </row>
@@ -43928,62 +43743,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>build</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>cFilesAnalyzed</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>creationDate</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>linesOfCode</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>linesOfComments</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>numberOfClasses</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>numberOfEntities</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>numberOfFiles</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>numberOfFunctions</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>systemFilesAnalyzed</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>taxonomies</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -43992,7 +43807,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>KW_Build_Label_Dec_04_2022_12_26_AM</t>
+          <t>KW_Build_Label_Feb_15_2023_12_21_PM</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
@@ -44000,26 +43815,26 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Sun Dec 04 01:05:35 IST 2022</t>
+          <t>Wed Feb 15 13:10:14 IST 2023</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>531520</v>
+        <v>532922</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>430758</v>
+        <v>430865</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>6518</v>
+        <v>6519</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>1000096</v>
+        <v>1000241</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>2524</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>11397</v>
+        <v>11413</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56</v>
@@ -44057,27 +43872,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>MISRA Metrics</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Default Range</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Number of Issues</t>
         </is>
@@ -44097,7 +43912,7 @@
       <c r="C2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Compiled</t>
         </is>
@@ -44120,7 +43935,7 @@
       <c r="C3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Compiled</t>
         </is>
@@ -44162,89 +43977,89 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Status: Ignore</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Status: Ignore without Waiver ID</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Status: Not a Problem</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Status: Not a Problem without Waiver ID</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>State: Existing</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>State: Existing AND need to be Analyzed or Fixed</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>State: New</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>State: New AND need to be Analyzed or Fixed</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Disapplied</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Permitted</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="L1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Permitted - Adopted Code</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Permitted - Module Specific</t>
         </is>
       </c>
-      <c r="N1" s="9" t="inlineStr">
+      <c r="N1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Permitted - Tool Issue</t>
         </is>
       </c>
-      <c r="O1" s="9" t="inlineStr">
+      <c r="O1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Tool Unsupported</t>
         </is>
       </c>
-      <c r="P1" s="9" t="inlineStr">
+      <c r="P1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: No plan to fix</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>MISRA Mandatory</t>
         </is>
@@ -44296,7 +44111,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>MISRA Required</t>
         </is>
@@ -44348,7 +44163,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>MISRA Advisory</t>
         </is>
@@ -44400,54 +44215,54 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="11" t="n">
+      <c r="B5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -44484,89 +44299,89 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Module name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Status: Ignore</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Status: Ignore without Waiver ID</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Status: Not a Problem</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Status: Not a Problem without Waiver ID</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>State: Existing</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>State: Existing AND need to be Analyzed or Fixed</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>State: New</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>State: New AND need to be Analyzed or Fixed</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Disapplied</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Permitted</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="L1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Permitted - Adopted Code</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Permitted - Module Specific</t>
         </is>
       </c>
-      <c r="N1" s="9" t="inlineStr">
+      <c r="N1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Permitted - Tool Issue</t>
         </is>
       </c>
-      <c r="O1" s="9" t="inlineStr">
+      <c r="O1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: Tool Unsupported</t>
         </is>
       </c>
-      <c r="P1" s="9" t="inlineStr">
+      <c r="P1" s="12" t="inlineStr">
         <is>
           <t>Deviation Type: No plan to fix</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>EthFw</t>
         </is>
@@ -44618,54 +44433,54 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="B3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="11" t="n">
+      <c r="B3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -44691,27 +44506,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>HIS Metrics</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Default Range</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Number of Issues</t>
         </is>
@@ -44733,7 +44548,7 @@
           <t>0-80</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Compiled</t>
         </is>
@@ -44758,7 +44573,7 @@
           <t>0-10</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Compiled</t>
         </is>
@@ -44783,7 +44598,7 @@
           <t>0-5</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Compiled</t>
         </is>
@@ -44808,7 +44623,7 @@
           <t>0-4</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Compiled</t>
         </is>
@@ -44818,15 +44633,15 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
-      <c r="E6" s="11" t="n">
+      <c r="B6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -44852,27 +44667,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Module name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Number of Paths</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Cyclomatic Complexity</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Number of Function Parameters</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Number of Call Levels</t>
         </is>
@@ -44898,21 +44713,21 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="B3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="11" t="n">
+      <c r="B3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -44946,74 +44761,74 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>State: New</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>State: New AND need to be Analyzed or Fixed</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>State: Existing</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>State: Existing AND need to be Analyzed or Fixed</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Status: Analyze</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Status: Ignore</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Status: Not a Problem</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Status: Defer</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Status: Fix</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Status: Fix in Next Release</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>Status: Fix in Later Release</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>Status: Filter</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>MISRA Mandatory</t>
         </is>
@@ -45056,7 +44871,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>MISRA Required</t>
         </is>
@@ -45099,7 +44914,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>MISRA Advisory</t>
         </is>
@@ -45142,7 +44957,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -45154,7 +44969,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>0</v>
@@ -45166,7 +44981,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>0</v>
@@ -45185,7 +45000,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Error</t>
         </is>
@@ -45197,7 +45012,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>0</v>
@@ -45209,7 +45024,7 @@
         <v>3</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>0</v>
@@ -45228,7 +45043,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Warning</t>
         </is>
@@ -45271,7 +45086,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
@@ -45314,7 +45129,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>HIS METRICS</t>
         </is>
@@ -45357,45 +45172,45 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="11" t="n">
+      <c r="B10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="E10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="11" t="n">
+      <c r="H10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="14" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ethfw: release docs update for 09.01.00 release
Signed-off-by: Sonu Alam <s-alam@ti.com>
</commit_message>
<xml_diff>
--- a/docs/misrac/ethfw_SA_Report.xlsx
+++ b/docs/misrac/ethfw_SA_Report.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Template Revision History" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="5" name="_xlnm._FilterDatabase">'Raw Issue Details'!$A$1:$O$10</definedName>
+    <definedName hidden="1" localSheetId="5" name="_xlnm._FilterDatabase">'Raw Issue Details'!$A$1:$O$9</definedName>
     <definedName hidden="1" localSheetId="6" name="_xlnm._FilterDatabase">'Taxonomy Checkers'!$A$1:$F$294</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -773,12 +773,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>ETHFW_KW_BUILD_Jul_19_2023_07_15_AM</t>
+          <t>ETHFW_KW_BUILD_Nov_22_2023_04_26_PM</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>status:'Not a Problem',Ignore severity:'Error','Critical'</t>
+          <t>severity:'Error','Critical'</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>2023-07-26 05:58:24.922948-05:00 CDT</t>
+          <t>2023-11-22 11:31:15.759823-06:00 CDT</t>
         </is>
       </c>
     </row>
@@ -885,37 +885,37 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>ETHFW_KW_BUILD_Jul_19_2023_07_15_AM</t>
+          <t>ETHFW_KW_BUILD_Nov_22_2023_04_26_PM</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1623</v>
+        <v>492</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Wed Jul 19 13:11:54 IST 2023</t>
+          <t>Wed Nov 22 22:37:40 IST 2023</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>275014</v>
+        <v>32785</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>281423</v>
+        <v>98448</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>5173</v>
+        <v>2475</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>253479</v>
+        <v>150495</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>1681</v>
+        <v>565</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>8680</v>
+        <v>876</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
@@ -1166,7 +1166,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>0</v>
@@ -1175,10 +1175,10 @@
         <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>0</v>
@@ -1209,7 +1209,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>0</v>
@@ -1218,7 +1218,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>2</v>
@@ -1381,7 +1381,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>0</v>
@@ -1390,10 +1390,10 @@
         <v>0</v>
       </c>
       <c r="G10" s="11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H10" s="11" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I10" s="11" t="n">
         <v>0</v>
@@ -1520,7 +1520,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>0</v>
@@ -1532,7 +1532,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -1563,7 +1563,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>0</v>
@@ -1572,10 +1572,10 @@
         <v>0</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>0</v>
@@ -1606,7 +1606,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4" s="11" t="n">
         <v>0</v>
@@ -1615,10 +1615,10 @@
         <v>0</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I4" s="11" t="n">
         <v>0</v>
@@ -1647,7 +1647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="18"/>
@@ -1752,33 +1752,29 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>INFINITE_LOOP.LOCAL</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Permitted by deviation: ID:PSDKRA_SA_DR_006</t>
-        </is>
-      </c>
+          <t>RH.LEAK</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr"/>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/ethremotecfg/server/src/remote_device_server_ethswitch.c</t>
+          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/utils/console_io/src/app_log_printf_ticgt_rtos.c</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>148377</v>
+        <v>1086257</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1376</v>
+        <v>243</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Infinite loop</t>
+          <t>Resource acquired to 'freopen("appLog:", "w", (&amp;_ftable[1]))' at line 243 may be lost here.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>rdevEthSwitchServerSenderTaskFn</t>
+          <t>appLogCioInit</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -1801,7 +1797,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Ignore</t>
+          <t>Not a Problem</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -1823,33 +1819,29 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ABV.STACK</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Specific EnetTypes are checked in lines 487-488 that would prevent the buffer overflow from happening.</t>
-        </is>
-      </c>
+          <t>INFINITE_LOOP.LOCAL</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr"/>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/ethfw/src/ethfw.c</t>
+          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/apps/app_remoteswitchcfg_server/mcu_2_0/main.c</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>423723</v>
+        <v>1087079</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1342</v>
+        <v>1529</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Array 'gMcmObj' of size 7 may use index value(s) 0..7</t>
+          <t>Infinite loop</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>EthFw_initMcm</t>
+          <t>EthApp_traceBufFlush</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -1859,11 +1851,11 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Error</t>
         </is>
       </c>
       <c r="J3" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
@@ -1887,40 +1879,40 @@
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>No Module</t>
+          <t>EthFw</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>INFINITE_LOOP.LOCAL</t>
+          <t>UNINIT.STACK.MUST</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>This is called by EthFw which runs forever and is not expected to be terminated.</t>
+          <t>Waiver id: PSDKRA_SA_DR_012</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/pdk_j7200_09_00_00_00/packages/ti/drv/enet/enet_cfgserver/enet_cfgserver.c</t>
+          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/utils/console_io/src/app_cli_rtos.c</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>700252</v>
+        <v>1240036</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>460</v>
+        <v>130</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Infinite loop</t>
+          <t>'args.__ap' is used uninitialized in this function.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>EnetCfgServer_networkTask</t>
+          <t>appCliPrintf</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -1930,11 +1922,11 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J4" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
@@ -1958,40 +1950,41 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>No Module</t>
+          <t>EthFw</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>INFINITE_LOOP.LOCAL</t>
+          <t>UNINIT.STACK.MUST</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>This is called by EthFw which runs forever and is not expected to be terminated.</t>
+          <t>Waiver id: PSDKRA_SA_DR_012
+reference: https://confluence.itg.ti.com/pages/viewpage.action?spaceKey=J7TDA4xSW&amp;title=PSDKRA+Static+Analysis+Policy</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/pdk_j7200_09_00_00_00/packages/ti/drv/enet/enet_cfgserver/enet_cfgserver.c</t>
+          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/apps/ipc_cfg/ipc_trace.c</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>700253</v>
+        <v>1240469</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>514</v>
+        <v>63</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Infinite loop</t>
+          <t>'args.__ap' is used uninitialized in this function.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>EnetCfgServer_dispatcherTask</t>
+          <t>Ipc_Trace_printf</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -2001,11 +1994,11 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J5" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
@@ -2029,40 +2022,40 @@
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>No Module</t>
+          <t>EthFw</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>RH.LEAK</t>
+          <t>UNINIT.STACK.MUST</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Permitted as per deviation record PSDKRA_SA_DR_011.</t>
+          <t>Waiver id: PSDKRA_SA_DR_012</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/utils/console_io/src/app_log_printf_ticgt_rtos.c</t>
+          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/apps/app_remoteswitchcfg_client/mcu_2_1/main.c</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1086257</v>
+        <v>1240569</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>243</v>
+        <v>499</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Resource acquired to 'freopen("appLog:", "w", (&amp;_ftable[1]))' at line 243 may be lost here.</t>
+          <t>'args.__ap' is used uninitialized in this function.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>appLogCioInit</t>
+          <t>appLogPrintf</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -2072,11 +2065,11 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J6" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
@@ -2085,7 +2078,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Ignore</t>
+          <t>Not a Problem</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -2107,33 +2100,34 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>INFINITE_LOOP.LOCAL</t>
+          <t>UNINIT.STACK.MUST</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Permitted as per deviation record PSDKRA_SA_DR_006.</t>
+          <t>Waiver id: PSDKRA_SA_DR_012
+reference: https://confluence.itg.ti.com/pages/viewpage.action?spaceKey=J7TDA4xSW&amp;title=PSDKRA+Static+Analysis+Policy</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/apps/app_remoteswitchcfg_server/mcu_2_0/main.c</t>
+          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/utils/console_io/src/app_log_writer.c</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1087079</v>
+        <v>1256325</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>1309</v>
+        <v>266</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Infinite loop</t>
+          <t>'va_args_ptr.__ap' is used uninitialized in this function.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>EthApp_traceBufFlush</t>
+          <t>appLogPrintf</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -2143,11 +2137,11 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J7" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
@@ -2156,7 +2150,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Ignore</t>
+          <t>Not a Problem</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -2183,28 +2177,29 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Waiver id: PSDKRA_SA_DR_012</t>
+          <t>Waiver id: PSDKRA_SA_DR_012
+reference: https://confluence.itg.ti.com/pages/viewpage.action?spaceKey=J7TDA4xSW&amp;title=PSDKRA+Static+Analysis+Policy</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/utils/console_io/src/app_cli_rtos.c</t>
+          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/utils/ethfw_common/src/ethfw_trace.c</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>1240036</v>
+        <v>1279934</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>130</v>
+        <v>272</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>'args.__ap' is used uninitialized in this function.</t>
+          <t>'ap.__ap' is used uninitialized in this function.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>appCliPrintf</t>
+          <t>EthFwTrace_trace</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -2254,19 +2249,20 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Waiver id: PSDKRA_SA_DR_012</t>
+          <t>Waiver id: PSDKRA_SA_DR_012
+reference: https://confluence.itg.ti.com/pages/viewpage.action?spaceKey=J7TDA4xSW&amp;title=PSDKRA+Static+Analysis+Policy</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/apps/ipc_cfg/ipc_trace.c</t>
+          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/utils/ethfw_common/src/ethfw_trace.c</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>1240469</v>
+        <v>1282473</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>63</v>
+        <v>205</v>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
@@ -2275,7 +2271,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Ipc_Trace_printf</t>
+          <t>EthFwTrace_print</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -2298,7 +2294,7 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Ignore</t>
+          <t>Not a Problem</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -2317,79 +2313,8 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>UNINIT.STACK.MUST</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Waiver id: PSDKRA_SA_DR_012</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>/nightlybuilds/repo_manifests/scripts/jenkins/workarea/ethfw/apps/app_remoteswitchcfg_client/mcu_2_1/main.c</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>1240569</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>476</v>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>'args.__ap' is used uninitialized in this function.</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>appLogPrintf</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>unowned</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t>Not a Problem</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="inlineStr">
-        <is>
-          <t>C and C++</t>
-        </is>
-      </c>
-      <c r="N10" s="3" t="inlineStr">
-        <is>
-          <t>KW Issue Link</t>
-        </is>
-      </c>
-      <c r="O10" s="3" t="inlineStr">
-        <is>
-          <t>EthFw</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O10"/>
+  <autoFilter ref="A1:O9"/>
   <hyperlinks>
     <hyperlink ref="N2" r:id="rId1"/>
     <hyperlink ref="N3" r:id="rId2"/>
@@ -2399,7 +2324,6 @@
     <hyperlink ref="N7" r:id="rId6"/>
     <hyperlink ref="N8" r:id="rId7"/>
     <hyperlink ref="N9" r:id="rId8"/>
-    <hyperlink ref="N10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>